<commit_message>
Semua ikon memakai Tabler Icons resmi; ikon sidebar satu color family dengan teks (aturan warna IDDS)
</commit_message>
<xml_diff>
--- a/Backlog-HE-EPPAT-Peruri.xlsx
+++ b/Backlog-HE-EPPAT-Peruri.xlsx
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3594" uniqueCount="2167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3600" uniqueCount="2171">
   <si>
     <t>Panduan Penerapan IDDS untuk Developer E-PPAT</t>
   </si>
@@ -6735,6 +6735,18 @@
   </si>
   <si>
     <t>prototipe/Backlog-HE-MINUTA-V2-Prototype.html; sumber/sidebar-seragam.js; semua prototipe tenant dan HE</t>
+  </si>
+  <si>
+    <t>Warna ikon menu samping disesuaikan dengan aturan warna IDDS (teks dan ikon memakai color family yang sama): ikon kini mengikuti warna teks menunya, yaitu putih redup saat biasa dan putih saat disorot atau aktif, menggantikan ikon emas #C2BB4B. Warna brand E-PPAT tetap tampil pada latar menu samping, menu aktif, dan kartu profil kantor. Uji kontras lulus.</t>
+  </si>
+  <si>
+    <t>sumber/order-idds.html; sumber/tera-idds.html; semua prototipe tenant dan HE</t>
+  </si>
+  <si>
+    <t>Semua ikon di luar menu samping (tombol, tabel, dialog, lencana, isian, kartu kantor, remah, dan index) diganti dengan Tabler Icons resmi versi 3.19.0, pustaka ikon IDDS. Sebanyak 112 jenis ikon dipetakan ke ikon Tabler yang paling dekat maknanya; audit isi SVG menunjukkan 0 ikon non-Tabler. Logo, ilustrasi, peta, kode QR, dan grafik tidak diubah.</t>
+  </si>
+  <si>
+    <t>sumber/aset/tabler-ui.json; sumber/ikon-tabler.js; semua prototipe</t>
   </si>
   <si>
     <t>Keterangan</t>
@@ -23212,7 +23224,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -24187,6 +24199,34 @@
       </c>
       <c r="D71" s="6" t="s">
         <v>2119</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="35">
+        <v>46322</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>1339</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>2120</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>2121</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="35">
+        <v>46322</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>2122</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>2123</v>
       </c>
     </row>
   </sheetData>
@@ -24210,19 +24250,19 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2120</v>
+        <v>2124</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>2121</v>
+        <v>2125</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="36" t="s">
-        <v>2122</v>
+        <v>2126</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>27</v>
@@ -24230,10 +24270,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
-        <v>2123</v>
+        <v>2127</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>2124</v>
+        <v>2128</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -24241,55 +24281,55 @@
         <v>1881</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>2125</v>
+        <v>2129</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
-        <v>2126</v>
+        <v>2130</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>2127</v>
+        <v>2131</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
-        <v>2128</v>
+        <v>2132</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>2129</v>
+        <v>2133</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
-        <v>2130</v>
+        <v>2134</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>2131</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
-        <v>2132</v>
+        <v>2136</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>2133</v>
+        <v>2137</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>2134</v>
+        <v>2138</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>2135</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
-        <v>2136</v>
+        <v>2140</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>2137</v>
+        <v>2141</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -24302,7 +24342,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>2138</v>
+        <v>2142</v>
       </c>
       <c r="B14" s="36" t="s">
         <v>27</v>
@@ -24310,26 +24350,26 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
-        <v>2139</v>
+        <v>2143</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>2140</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
-        <v>2141</v>
+        <v>2145</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>2142</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>2143</v>
+        <v>2147</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>2144</v>
+        <v>2148</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -24337,7 +24377,7 @@
         <v>517</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>2145</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -24345,7 +24385,7 @@
         <v>8</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>2146</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -24369,7 +24409,7 @@
         <v>1886</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>2147</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -24377,7 +24417,7 @@
         <v>541</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>2148</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -24385,7 +24425,7 @@
         <v>550</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>2149</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -24393,7 +24433,7 @@
         <v>1887</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>2150</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -24401,7 +24441,7 @@
         <v>1888</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>2151</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -24409,7 +24449,7 @@
         <v>1889</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>2152</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -24417,7 +24457,7 @@
         <v>1890</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>2153</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -24430,7 +24470,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="36" t="s">
-        <v>2154</v>
+        <v>2158</v>
       </c>
       <c r="B30" s="36" t="s">
         <v>27</v>
@@ -24438,7 +24478,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
-        <v>2155</v>
+        <v>2159</v>
       </c>
       <c r="B31" s="37" t="s">
         <v>1933</v>
@@ -24446,7 +24486,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
-        <v>2156</v>
+        <v>2160</v>
       </c>
       <c r="B32" s="37" t="s">
         <v>1935</v>
@@ -24454,7 +24494,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="37" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
       <c r="B33" s="37" t="s">
         <v>1937</v>
@@ -24462,7 +24502,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="37" t="s">
-        <v>2158</v>
+        <v>2162</v>
       </c>
       <c r="B34" s="37" t="s">
         <v>1939</v>
@@ -24470,15 +24510,15 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="37" t="s">
-        <v>2159</v>
+        <v>2163</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>2160</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="37" t="s">
-        <v>2161</v>
+        <v>2165</v>
       </c>
       <c r="B36" s="37" t="s">
         <v>1943</v>
@@ -24486,7 +24526,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="37" t="s">
-        <v>2162</v>
+        <v>2166</v>
       </c>
       <c r="B37" s="37" t="s">
         <v>1945</v>
@@ -24494,7 +24534,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="37" t="s">
-        <v>2163</v>
+        <v>2167</v>
       </c>
       <c r="B38" s="37" t="s">
         <v>1947</v>
@@ -24502,7 +24542,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="37" t="s">
-        <v>2164</v>
+        <v>2168</v>
       </c>
       <c r="B39" s="37" t="s">
         <v>1949</v>
@@ -24510,7 +24550,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="37" t="s">
-        <v>2165</v>
+        <v>2169</v>
       </c>
       <c r="B40" s="37" t="s">
         <v>1951</v>
@@ -24518,7 +24558,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="37" t="s">
-        <v>2166</v>
+        <v>2170</v>
       </c>
       <c r="B41" s="37" t="s">
         <v>1953</v>

</xml_diff>

<commit_message>
Penyusunan Akta v2: sidebar otomatis ciut di editor; ikon catatan Tabler pilcrow; latar polos tema INAgov/Default; riwayat xlsx
</commit_message>
<xml_diff>
--- a/Backlog-HE-EPPAT-Peruri.xlsx
+++ b/Backlog-HE-EPPAT-Peruri.xlsx
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3625" uniqueCount="2188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="2192">
   <si>
     <t>Panduan Penerapan IDDS untuk Developer E-PPAT</t>
   </si>
@@ -6798,6 +6798,18 @@
   </si>
   <si>
     <t>sumber/tema-proto.html; sumber/rakit-idds.js; prototipe/Backlog-IDDS-TN-CMS-Prototype.html; Backlog-IDDS-PL-SISTEM-Prototype.html; semua prototipe</t>
+  </si>
+  <si>
+    <t>Tema INAgov dan Default memakai latar polos netral IDDS (--ina-background-secondary) di semua halaman, termasuk halaman Masuk tenant dan platform. Latar bergambar khas E-PPAT (gradasi dengan watermark IPPAT) hanya dipakai tema E-PPAT. Token warna INAgov dan Default sudah dicocokkan dengan CSS resmi IDDS 1.6.38 (0 perbedaan).</t>
+  </si>
+  <si>
+    <t>sumber/tema-proto.html; semua prototipe</t>
+  </si>
+  <si>
+    <t>Saat pengguna membuka editor Penyusunan Akta v2, menu samping otomatis diciutkan menjadi ikon (72 px) agar kertas lebih lega. Saat kembali ke daftar, menu samping mengikuti pilihan terakhir pengguna. Ciut otomatis ini tidak menimpa pilihan tersimpan dan tidak berlaku di ponsel karena menu samping sudah berupa laci. Ikon catatan pada Navigasi diganti dengan ikon Tabler pilcrow.</t>
+  </si>
+  <si>
+    <t>sumber/sidebar-idds.html; sumber/minuta2-badan.html; prototipe/Backlog-HE-MINUTA-V2-Prototype.html; semua prototipe bersidebar</t>
   </si>
   <si>
     <t>Keterangan</t>
@@ -23369,7 +23381,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -24386,6 +24398,34 @@
       </c>
       <c r="D74" s="6" t="s">
         <v>2140</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" s="35">
+        <v>46322</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>2138</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>2141</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>2142</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="35">
+        <v>46323</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>712</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>2143</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>2144</v>
       </c>
     </row>
   </sheetData>
@@ -24409,19 +24449,19 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2141</v>
+        <v>2145</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>2142</v>
+        <v>2146</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="36" t="s">
-        <v>2143</v>
+        <v>2147</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>27</v>
@@ -24429,10 +24469,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
-        <v>2144</v>
+        <v>2148</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>2145</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -24440,55 +24480,55 @@
         <v>1895</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>2146</v>
+        <v>2150</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
-        <v>2147</v>
+        <v>2151</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>2148</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
-        <v>2149</v>
+        <v>2153</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>2150</v>
+        <v>2154</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
-        <v>2151</v>
+        <v>2155</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>2152</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
-        <v>2153</v>
+        <v>2157</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>2154</v>
+        <v>2158</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>2155</v>
+        <v>2159</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>2156</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
-        <v>2157</v>
+        <v>2161</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>2158</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -24501,7 +24541,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>2159</v>
+        <v>2163</v>
       </c>
       <c r="B14" s="36" t="s">
         <v>27</v>
@@ -24509,26 +24549,26 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
-        <v>2160</v>
+        <v>2164</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>2161</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
-        <v>2162</v>
+        <v>2166</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>2163</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>2164</v>
+        <v>2168</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>2165</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -24536,7 +24576,7 @@
         <v>517</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>2166</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -24544,7 +24584,7 @@
         <v>8</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>2167</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -24568,7 +24608,7 @@
         <v>1900</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>2168</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -24576,7 +24616,7 @@
         <v>541</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>2169</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -24584,7 +24624,7 @@
         <v>550</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -24592,7 +24632,7 @@
         <v>1901</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>2171</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -24600,7 +24640,7 @@
         <v>1902</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>2172</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -24608,7 +24648,7 @@
         <v>1903</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>2173</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -24616,7 +24656,7 @@
         <v>1904</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>2174</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -24629,7 +24669,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="36" t="s">
-        <v>2175</v>
+        <v>2179</v>
       </c>
       <c r="B30" s="36" t="s">
         <v>27</v>
@@ -24637,7 +24677,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
-        <v>2176</v>
+        <v>2180</v>
       </c>
       <c r="B31" s="37" t="s">
         <v>1947</v>
@@ -24645,7 +24685,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
-        <v>2177</v>
+        <v>2181</v>
       </c>
       <c r="B32" s="37" t="s">
         <v>1949</v>
@@ -24653,7 +24693,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="37" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
       <c r="B33" s="37" t="s">
         <v>1951</v>
@@ -24661,7 +24701,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="37" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="B34" s="37" t="s">
         <v>1953</v>
@@ -24669,15 +24709,15 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="37" t="s">
-        <v>2180</v>
+        <v>2184</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>2181</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="37" t="s">
-        <v>2182</v>
+        <v>2186</v>
       </c>
       <c r="B36" s="37" t="s">
         <v>1957</v>
@@ -24685,7 +24725,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="37" t="s">
-        <v>2183</v>
+        <v>2187</v>
       </c>
       <c r="B37" s="37" t="s">
         <v>1959</v>
@@ -24693,7 +24733,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="37" t="s">
-        <v>2184</v>
+        <v>2188</v>
       </c>
       <c r="B38" s="37" t="s">
         <v>1961</v>
@@ -24701,7 +24741,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="37" t="s">
-        <v>2185</v>
+        <v>2189</v>
       </c>
       <c r="B39" s="37" t="s">
         <v>1963</v>
@@ -24709,7 +24749,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="37" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="B40" s="37" t="s">
         <v>1965</v>
@@ -24717,7 +24757,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="37" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="B41" s="37" t="s">
         <v>1967</v>

</xml_diff>

<commit_message>
Header: tombol menu hanya di layar sempit; layar lebar pakai tombol ciut sidebar; riwayat xlsx
</commit_message>
<xml_diff>
--- a/Backlog-HE-EPPAT-Peruri.xlsx
+++ b/Backlog-HE-EPPAT-Peruri.xlsx
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3631" uniqueCount="2192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3634" uniqueCount="2195">
   <si>
     <t>Panduan Penerapan IDDS untuk Developer E-PPAT</t>
   </si>
@@ -6810,6 +6810,15 @@
   </si>
   <si>
     <t>sumber/sidebar-idds.html; sumber/minuta2-badan.html; prototipe/Backlog-HE-MINUTA-V2-Prototype.html; semua prototipe bersidebar</t>
+  </si>
+  <si>
+    <t>IDDS-TN-40; IDDS-PL-41</t>
+  </si>
+  <si>
+    <t>Tombol menu (ikon tiga garis) di header kini hanya tampil di layar sempit untuk membuka laci menu samping. Di layar lebar tombol itu disembunyikan karena tidak berfungsi; menu samping diciutkan atau dibentangkan dengan tombol di kepala menu samping. Dengan begitu, setiap ukuran layar hanya punya satu kendali menu samping.</t>
+  </si>
+  <si>
+    <t>sumber/sidebar-idds.html; semua prototipe bersidebar</t>
   </si>
   <si>
     <t>Keterangan</t>
@@ -23381,7 +23390,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -24426,6 +24435,20 @@
       </c>
       <c r="D76" s="6" t="s">
         <v>2144</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="35">
+        <v>46323</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>2145</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>2146</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>2147</v>
       </c>
     </row>
   </sheetData>
@@ -24449,19 +24472,19 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2145</v>
+        <v>2148</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>2146</v>
+        <v>2149</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="36" t="s">
-        <v>2147</v>
+        <v>2150</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>27</v>
@@ -24469,10 +24492,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
-        <v>2148</v>
+        <v>2151</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>2149</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -24480,55 +24503,55 @@
         <v>1895</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>2150</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
-        <v>2151</v>
+        <v>2154</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>2152</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
-        <v>2153</v>
+        <v>2156</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>2154</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
-        <v>2155</v>
+        <v>2158</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>2156</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
-        <v>2157</v>
+        <v>2160</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>2158</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>2159</v>
+        <v>2162</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>2160</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
-        <v>2161</v>
+        <v>2164</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>2162</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -24541,7 +24564,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="36" t="s">
-        <v>2163</v>
+        <v>2166</v>
       </c>
       <c r="B14" s="36" t="s">
         <v>27</v>
@@ -24549,26 +24572,26 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
-        <v>2164</v>
+        <v>2167</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>2167</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>2168</v>
+        <v>2171</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>2169</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -24576,7 +24599,7 @@
         <v>517</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>2170</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -24584,7 +24607,7 @@
         <v>8</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>2171</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -24608,7 +24631,7 @@
         <v>1900</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>2172</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -24616,7 +24639,7 @@
         <v>541</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>2173</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -24624,7 +24647,7 @@
         <v>550</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>2174</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -24632,7 +24655,7 @@
         <v>1901</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>2175</v>
+        <v>2178</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -24640,7 +24663,7 @@
         <v>1902</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>2176</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -24648,7 +24671,7 @@
         <v>1903</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>2177</v>
+        <v>2180</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -24656,7 +24679,7 @@
         <v>1904</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>2178</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -24669,7 +24692,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="36" t="s">
-        <v>2179</v>
+        <v>2182</v>
       </c>
       <c r="B30" s="36" t="s">
         <v>27</v>
@@ -24677,7 +24700,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
-        <v>2180</v>
+        <v>2183</v>
       </c>
       <c r="B31" s="37" t="s">
         <v>1947</v>
@@ -24685,7 +24708,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
-        <v>2181</v>
+        <v>2184</v>
       </c>
       <c r="B32" s="37" t="s">
         <v>1949</v>
@@ -24693,7 +24716,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="37" t="s">
-        <v>2182</v>
+        <v>2185</v>
       </c>
       <c r="B33" s="37" t="s">
         <v>1951</v>
@@ -24701,7 +24724,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="37" t="s">
-        <v>2183</v>
+        <v>2186</v>
       </c>
       <c r="B34" s="37" t="s">
         <v>1953</v>
@@ -24709,15 +24732,15 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="37" t="s">
-        <v>2184</v>
+        <v>2187</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>2185</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="37" t="s">
-        <v>2186</v>
+        <v>2189</v>
       </c>
       <c r="B36" s="37" t="s">
         <v>1957</v>
@@ -24725,7 +24748,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="37" t="s">
-        <v>2187</v>
+        <v>2190</v>
       </c>
       <c r="B37" s="37" t="s">
         <v>1959</v>
@@ -24733,7 +24756,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="37" t="s">
-        <v>2188</v>
+        <v>2191</v>
       </c>
       <c r="B38" s="37" t="s">
         <v>1961</v>
@@ -24741,7 +24764,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="37" t="s">
-        <v>2189</v>
+        <v>2192</v>
       </c>
       <c r="B39" s="37" t="s">
         <v>1963</v>
@@ -24749,7 +24772,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="37" t="s">
-        <v>2190</v>
+        <v>2193</v>
       </c>
       <c r="B40" s="37" t="s">
         <v>1965</v>
@@ -24757,7 +24780,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="37" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="B41" s="37" t="s">
         <v>1967</v>

</xml_diff>